<commit_message>
docs: add QA traceability, defect register, test plan, and verification report artifacts
</commit_message>
<xml_diff>
--- a/grc_wisdom_api/scripts/verify/_tmp/Audit_report.xlsx
+++ b/grc_wisdom_api/scripts/verify/_tmp/Audit_report.xlsx
@@ -49,7 +49,7 @@
     <t>Generated at</t>
   </si>
   <si>
-    <t>2026-09-23 10:59 UTC</t>
+    <t>2026-09-24 22:36 UTC</t>
   </si>
   <si>
     <t>Visibility</t>
@@ -61,7 +61,7 @@
     <t>Document reference</t>
   </si>
   <si>
-    <t>1172-20260923105942</t>
+    <t>97EF-20260924223621</t>
   </si>
   <si>
     <t>DRAFT — this engagement is Planned. Figures are provisional and the conclusion is not final.</t>
@@ -82,7 +82,7 @@
     <t>Lead auditor</t>
   </si>
   <si>
-    <t>Shahd Hamdan</t>
+    <t>Mehdi Tantaoui</t>
   </si>
   <si>
     <t>Status</t>

</xml_diff>